<commit_message>
a random thingy for getting the data
</commit_message>
<xml_diff>
--- a/RMSE_MetalAbenics.xlsx
+++ b/RMSE_MetalAbenics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SWP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SWP\SRA_Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1617DB8-AD35-4D2F-AEA7-A1A14D2A9AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96EFA3F-6D15-4702-87CC-0C7CF0E16371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{173C258E-E726-4BC5-B9C3-67A262576D29}"/>
   </bookViews>
@@ -413,75 +413,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFD8B15B-CD9D-4BFF-814C-4BA5ED592BD9}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
+        <v>1.0989391224927101</v>
+      </c>
+      <c r="C3">
         <v>0.39304865472140899</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
+        <v>1.1538272385569199</v>
+      </c>
+      <c r="C4">
         <v>0.11746224969781199</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
+        <v>2.13906892190957</v>
+      </c>
+      <c r="C5">
         <v>0.302306789652664</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6">
+        <v>3.0364896195594899</v>
+      </c>
+      <c r="C6">
         <v>0.39808986944745001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
+        <v>1.77406295008255</v>
+      </c>
+      <c r="C7">
         <v>0.15723183253658199</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
+        <v>1.7328968630343899</v>
+      </c>
+      <c r="C8">
         <v>0.213245329492598</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9">
+        <v>2.5973846910457699</v>
+      </c>
+      <c r="C9">
         <v>0.49331281427267698</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10">
+        <v>1.54902167421927</v>
+      </c>
+      <c r="C10">
         <v>0.60253913333690801</v>
       </c>
     </row>

</xml_diff>